<commit_message>
Grandes Atualizações e inclusão da calculadora de comissões (método padrão utilizado pela Ana hoje)
</commit_message>
<xml_diff>
--- a/Comissoes_Recebimento_10_2025.xlsx
+++ b/Comissoes_Recebimento_10_2025.xlsx
@@ -19,9 +19,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -38,7 +36,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -49,6 +47,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="0037474F"/>
         <bgColor rgb="0037474F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F8E9"/>
+        <bgColor rgb="00F1F8E9"/>
       </patternFill>
     </fill>
   </fills>
@@ -70,16 +74,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -462,57 +465,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>processo</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>documento</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>data_pagamento</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>valor_pago</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>nome_colaborador</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>cargo</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>tcmp</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>fc</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>comissao_calculada</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>mes_calculo</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>observacao</t>
         </is>
@@ -529,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -540,71 +543,187 @@
     <col width="7" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
     <col width="6" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>processo</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>documento</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>data_pagamento</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>valor_pago</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>nome_colaborador</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>cargo</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>tcmp</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>fc</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>fcmp</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>comissao_calculada</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>tipo_lancamento</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>mes_faturamento</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>mes_calculo</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
-        <is>
-          <t>observacao</t>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>TESTE</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>999001</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>15/10/2025</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>40.00</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>André Caramello</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr"/>
+      <c r="G2" s="3" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H2" s="3" t="inlineStr"/>
+      <c r="I2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>0.40</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>Pagamento Regular</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>10/2025</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>10/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>TESTE2</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>999002</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>20/10/2025</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>30.00</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>André Caramello</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H3" s="3" t="inlineStr"/>
+      <c r="I3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>0.30</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Pagamento Regular</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>10/2025</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>10/2025</t>
         </is>
       </c>
     </row>
@@ -634,47 +753,47 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>processo</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>colaborador</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>tcmp</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>fcmp</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>comissao_adiantada_fc_1</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>comissao_deveria_fc_real</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>diferenca_fc</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>ajuste_reconciliacao</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>mes_faturamento</t>
         </is>
@@ -691,87 +810,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>documento</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>documento_6dig</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>motivo</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>valor</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>data_pagamento</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>999001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>999001</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>NF não encontrada na Análise Comercial: 999001</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>40</v>
-      </c>
-      <c r="E2" s="4" t="n">
-        <v>45945</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>999002</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>999002</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>NF não encontrada na Análise Comercial: 999002</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>30</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>45950</v>
       </c>
     </row>
   </sheetData>

</xml_diff>